<commit_message>
Actualizar datos 2026 (2026-04-14)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>35.02%</t>
+    <t>36.35%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
   </si>
   <si>
-    <t>55.06%</t>
+    <t>57.30%</t>
   </si>
   <si>
     <t>General 1ra Base</t>
@@ -103,6 +103,12 @@
     <t>2.19%</t>
   </si>
   <si>
+    <t>Parrilladas</t>
+  </si>
+  <si>
+    <t>0.00%</t>
+  </si>
+  <si>
     <t>Personas con Discapacidad</t>
   </si>
   <si>
@@ -112,19 +118,19 @@
     <t>VIP</t>
   </si>
   <si>
-    <t>75.82%</t>
+    <t>77.72%</t>
   </si>
   <si>
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>39.13%</t>
+    <t>41.21%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>24.73%</t>
+    <t>24.88%</t>
   </si>
 </sst>
 </file>
@@ -546,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -637,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -676,10 +682,10 @@
         <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="Q6" s="6">
-        <v>538</v>
+        <v>527</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -693,7 +699,7 @@
         <v>534</v>
       </c>
       <c r="C7" s="6">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -732,10 +738,10 @@
         <v>7</v>
       </c>
       <c r="P7" s="6">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="Q7" s="6">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -858,7 +864,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="6">
-        <v>27</v>
+        <v>180</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>22</v>
@@ -872,8 +878,8 @@
       <c r="F10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="6">
-        <v>1</v>
+      <c r="G10" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>22</v>
@@ -899,11 +905,11 @@
       <c r="O10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="P10" s="6">
-        <v>1</v>
+      <c r="P10" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="Q10" s="6">
-        <v>26</v>
+        <v>180</v>
       </c>
       <c r="R10" s="6" t="s">
         <v>31</v>
@@ -914,34 +920,34 @@
         <v>32</v>
       </c>
       <c r="B11" s="6">
-        <v>368</v>
-      </c>
-      <c r="C11" s="6">
-        <v>63</v>
+        <v>27</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="6">
-        <v>50</v>
+      <c r="E11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="G11" s="6">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="6">
-        <v>57</v>
+      <c r="I11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="K11" s="6">
-        <v>2</v>
+      <c r="K11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>22</v>
@@ -949,17 +955,17 @@
       <c r="M11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="N11" s="6">
-        <v>78</v>
+      <c r="N11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P11" s="6">
-        <v>279</v>
+        <v>1</v>
       </c>
       <c r="Q11" s="6">
-        <v>89</v>
+        <v>26</v>
       </c>
       <c r="R11" s="6" t="s">
         <v>33</v>
@@ -970,34 +976,34 @@
         <v>34</v>
       </c>
       <c r="B12" s="6">
-        <v>1109</v>
+        <v>368</v>
       </c>
       <c r="C12" s="6">
-        <v>224</v>
+        <v>65</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="G12" s="6">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I12" s="6">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="K12" s="6">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="L12" s="6" t="s">
         <v>22</v>
@@ -1006,79 +1012,135 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>434</v>
+        <v>286</v>
       </c>
       <c r="Q12" s="6">
-        <v>675</v>
+        <v>82</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="7">
-        <f>SUM(B6:B12)</f>
-      </c>
-      <c r="C13" s="7">
-        <f>SUM(C6:C12)</f>
-      </c>
-      <c r="D13" s="7">
-        <f>SUM(D6:D12)</f>
-      </c>
-      <c r="E13" s="7">
-        <f>SUM(E6:E12)</f>
-      </c>
-      <c r="F13" s="7">
-        <f>SUM(F6:F12)</f>
-      </c>
-      <c r="G13" s="7">
-        <f>SUM(G6:G12)</f>
-      </c>
-      <c r="H13" s="7">
-        <f>SUM(H6:H12)</f>
-      </c>
-      <c r="I13" s="7">
-        <f>SUM(I6:I12)</f>
-      </c>
-      <c r="J13" s="7">
-        <f>SUM(J6:J12)</f>
-      </c>
-      <c r="K13" s="7">
-        <f>SUM(K6:K12)</f>
-      </c>
-      <c r="L13" s="7">
-        <f>SUM(L6:L12)</f>
-      </c>
-      <c r="M13" s="7">
-        <f>SUM(M6:M12)</f>
-      </c>
-      <c r="N13" s="7">
-        <f>SUM(N6:N12)</f>
-      </c>
-      <c r="O13" s="7">
-        <f>SUM(O6:O12)</f>
-      </c>
-      <c r="P13" s="7">
-        <f>SUM(P6:P12)</f>
-      </c>
-      <c r="Q13" s="7">
-        <f>SUM(Q6:Q12)</f>
-      </c>
-      <c r="R13" s="7" t="s">
+      <c r="B13" s="6">
+        <v>1109</v>
+      </c>
+      <c r="C13" s="6">
+        <v>241</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="6">
+        <v>65</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="6">
+        <v>32</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="6">
+        <v>49</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K13" s="6">
+        <v>26</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="N13" s="6">
+        <v>44</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P13" s="6">
+        <v>457</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>652</v>
+      </c>
+      <c r="R13" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="7">
+        <f>SUM(B6:B13)</f>
+      </c>
+      <c r="C14" s="7">
+        <f>SUM(C6:C13)</f>
+      </c>
+      <c r="D14" s="7">
+        <f>SUM(D6:D13)</f>
+      </c>
+      <c r="E14" s="7">
+        <f>SUM(E6:E13)</f>
+      </c>
+      <c r="F14" s="7">
+        <f>SUM(F6:F13)</f>
+      </c>
+      <c r="G14" s="7">
+        <f>SUM(G6:G13)</f>
+      </c>
+      <c r="H14" s="7">
+        <f>SUM(H6:H13)</f>
+      </c>
+      <c r="I14" s="7">
+        <f>SUM(I6:I13)</f>
+      </c>
+      <c r="J14" s="7">
+        <f>SUM(J6:J13)</f>
+      </c>
+      <c r="K14" s="7">
+        <f>SUM(K6:K13)</f>
+      </c>
+      <c r="L14" s="7">
+        <f>SUM(L6:L13)</f>
+      </c>
+      <c r="M14" s="7">
+        <f>SUM(M6:M13)</f>
+      </c>
+      <c r="N14" s="7">
+        <f>SUM(N6:N13)</f>
+      </c>
+      <c r="O14" s="7">
+        <f>SUM(O6:O13)</f>
+      </c>
+      <c r="P14" s="7">
+        <f>SUM(P6:P13)</f>
+      </c>
+      <c r="Q14" s="7">
+        <f>SUM(Q6:Q13)</f>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar datos 2026 (2026-04-15)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>36.35%</t>
+    <t>39.73%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
   </si>
   <si>
-    <t>57.30%</t>
+    <t>57.87%</t>
   </si>
   <si>
     <t>General 1ra Base</t>
@@ -118,19 +118,19 @@
     <t>VIP</t>
   </si>
   <si>
-    <t>77.72%</t>
+    <t>78.80%</t>
   </si>
   <si>
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>41.21%</t>
+    <t>43.10%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>24.88%</t>
+    <t>25.88%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -682,10 +682,10 @@
         <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>301</v>
+        <v>329</v>
       </c>
       <c r="Q6" s="6">
-        <v>527</v>
+        <v>499</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +699,7 @@
         <v>534</v>
       </c>
       <c r="C7" s="6">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -723,7 +723,7 @@
         <v>22</v>
       </c>
       <c r="K7" s="6">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>22</v>
@@ -738,10 +738,10 @@
         <v>7</v>
       </c>
       <c r="P7" s="6">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="Q7" s="6">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -1012,16 +1012,16 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="Q12" s="6">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>35</v>
@@ -1035,7 +1035,7 @@
         <v>1109</v>
       </c>
       <c r="C13" s="6">
-        <v>241</v>
+        <v>264</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
@@ -1059,7 +1059,7 @@
         <v>22</v>
       </c>
       <c r="K13" s="6">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>22</v>
@@ -1068,16 +1068,16 @@
         <v>22</v>
       </c>
       <c r="N13" s="6">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P13" s="6">
-        <v>457</v>
+        <v>478</v>
       </c>
       <c r="Q13" s="6">
-        <v>652</v>
+        <v>631</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Actualizar datos 2026 (2026-04-16)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>39.73%</t>
+    <t>41.06%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
   </si>
   <si>
-    <t>57.87%</t>
+    <t>58.24%</t>
   </si>
   <si>
     <t>General 1ra Base</t>
@@ -124,13 +124,13 @@
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>43.10%</t>
+    <t>44.18%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>25.88%</t>
+    <t>26.33%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -682,10 +682,10 @@
         <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="Q6" s="6">
-        <v>499</v>
+        <v>488</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +699,7 @@
         <v>534</v>
       </c>
       <c r="C7" s="6">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -738,10 +738,10 @@
         <v>7</v>
       </c>
       <c r="P7" s="6">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="Q7" s="6">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -1035,7 +1035,7 @@
         <v>1109</v>
       </c>
       <c r="C13" s="6">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
@@ -1074,10 +1074,10 @@
         <v>22</v>
       </c>
       <c r="P13" s="6">
-        <v>478</v>
+        <v>490</v>
       </c>
       <c r="Q13" s="6">
-        <v>631</v>
+        <v>619</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Actualizar datos 2026 (2026-04-16 PM)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,25 +82,25 @@
     <t>-</t>
   </si>
   <si>
-    <t>41.06%</t>
+    <t>46.01%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
   </si>
   <si>
-    <t>58.24%</t>
+    <t>49.44%</t>
   </si>
   <si>
     <t>General 1ra Base</t>
   </si>
   <si>
-    <t>0.74%</t>
+    <t>0.82%</t>
   </si>
   <si>
     <t>General 3ra Base</t>
   </si>
   <si>
-    <t>2.19%</t>
+    <t>3.02%</t>
   </si>
   <si>
     <t>Parrilladas</t>
@@ -124,13 +124,13 @@
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>44.18%</t>
+    <t>47.61%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>26.33%</t>
+    <t>27.12%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -667,7 +667,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="6">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>22</v>
@@ -676,16 +676,16 @@
         <v>22</v>
       </c>
       <c r="N6" s="6">
-        <v>43</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>22</v>
+        <v>69</v>
+      </c>
+      <c r="O6" s="6">
+        <v>2</v>
       </c>
       <c r="P6" s="6">
-        <v>340</v>
+        <v>381</v>
       </c>
       <c r="Q6" s="6">
-        <v>488</v>
+        <v>447</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +699,7 @@
         <v>534</v>
       </c>
       <c r="C7" s="6">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -732,16 +732,16 @@
         <v>22</v>
       </c>
       <c r="N7" s="6">
-        <v>157</v>
+        <v>107</v>
       </c>
       <c r="O7" s="6">
         <v>7</v>
       </c>
       <c r="P7" s="6">
-        <v>311</v>
+        <v>264</v>
       </c>
       <c r="Q7" s="6">
-        <v>223</v>
+        <v>270</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -767,7 +767,7 @@
         <v>22</v>
       </c>
       <c r="G8" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>22</v>
@@ -794,10 +794,10 @@
         <v>22</v>
       </c>
       <c r="P8" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="6">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="R8" s="6" t="s">
         <v>27</v>
@@ -811,7 +811,7 @@
         <v>1324</v>
       </c>
       <c r="C9" s="6">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>22</v>
@@ -850,10 +850,10 @@
         <v>22</v>
       </c>
       <c r="P9" s="6">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="Q9" s="6">
-        <v>1295</v>
+        <v>1284</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
@@ -1035,13 +1035,13 @@
         <v>1109</v>
       </c>
       <c r="C13" s="6">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="6">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>22</v>
@@ -1068,16 +1068,16 @@
         <v>22</v>
       </c>
       <c r="N13" s="6">
-        <v>40</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>22</v>
+        <v>43</v>
+      </c>
+      <c r="O13" s="6">
+        <v>3</v>
       </c>
       <c r="P13" s="6">
-        <v>490</v>
+        <v>528</v>
       </c>
       <c r="Q13" s="6">
-        <v>619</v>
+        <v>581</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Actualizar datos 2026 (2026-04-17)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,25 +82,25 @@
     <t>-</t>
   </si>
   <si>
-    <t>46.01%</t>
+    <t>49.76%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
   </si>
   <si>
-    <t>49.44%</t>
+    <t>50.19%</t>
   </si>
   <si>
     <t>General 1ra Base</t>
   </si>
   <si>
-    <t>0.82%</t>
+    <t>0.91%</t>
   </si>
   <si>
     <t>General 3ra Base</t>
   </si>
   <si>
-    <t>3.02%</t>
+    <t>3.55%</t>
   </si>
   <si>
     <t>Parrilladas</t>
@@ -118,19 +118,19 @@
     <t>VIP</t>
   </si>
   <si>
-    <t>78.80%</t>
+    <t>81.52%</t>
   </si>
   <si>
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>47.61%</t>
+    <t>50.05%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>27.12%</t>
+    <t>28.55%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>210</v>
+        <v>236</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -667,7 +667,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="6">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>22</v>
@@ -679,13 +679,13 @@
         <v>69</v>
       </c>
       <c r="O6" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P6" s="6">
-        <v>381</v>
+        <v>412</v>
       </c>
       <c r="Q6" s="6">
-        <v>447</v>
+        <v>416</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +699,7 @@
         <v>534</v>
       </c>
       <c r="C7" s="6">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -738,10 +738,10 @@
         <v>7</v>
       </c>
       <c r="P7" s="6">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="Q7" s="6">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -755,7 +755,7 @@
         <v>1213</v>
       </c>
       <c r="C8" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>22</v>
@@ -794,10 +794,10 @@
         <v>22</v>
       </c>
       <c r="P8" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q8" s="6">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="R8" s="6" t="s">
         <v>27</v>
@@ -817,7 +817,7 @@
         <v>22</v>
       </c>
       <c r="E9" s="6">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>22</v>
@@ -850,10 +850,10 @@
         <v>22</v>
       </c>
       <c r="P9" s="6">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="Q9" s="6">
-        <v>1284</v>
+        <v>1277</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
@@ -985,7 +985,7 @@
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
@@ -1012,16 +1012,16 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="Q12" s="6">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>35</v>
@@ -1035,7 +1035,7 @@
         <v>1109</v>
       </c>
       <c r="C13" s="6">
-        <v>283</v>
+        <v>312</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
@@ -1053,7 +1053,7 @@
         <v>22</v>
       </c>
       <c r="I13" s="6">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>22</v>
@@ -1070,14 +1070,14 @@
       <c r="N13" s="6">
         <v>43</v>
       </c>
-      <c r="O13" s="6">
-        <v>3</v>
+      <c r="O13" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P13" s="6">
-        <v>528</v>
+        <v>555</v>
       </c>
       <c r="Q13" s="6">
-        <v>581</v>
+        <v>554</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Actualizar datos 2026 (2026-04-17 PM)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -82,7 +82,7 @@
     <t>-</t>
   </si>
   <si>
-    <t>49.76%</t>
+    <t>51.21%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
@@ -118,19 +118,19 @@
     <t>VIP</t>
   </si>
   <si>
-    <t>81.52%</t>
+    <t>82.88%</t>
   </si>
   <si>
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>50.05%</t>
+    <t>55.64%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>28.55%</t>
+    <t>29.97%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -678,14 +678,14 @@
       <c r="N6" s="6">
         <v>69</v>
       </c>
-      <c r="O6" s="6">
-        <v>4</v>
+      <c r="O6" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="Q6" s="6">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -979,13 +979,13 @@
         <v>368</v>
       </c>
       <c r="C12" s="6">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
@@ -1018,10 +1018,10 @@
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="Q12" s="6">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>35</v>
@@ -1035,13 +1035,13 @@
         <v>1109</v>
       </c>
       <c r="C13" s="6">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="6">
-        <v>90</v>
+        <v>131</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>22</v>
@@ -1070,14 +1070,14 @@
       <c r="N13" s="6">
         <v>43</v>
       </c>
-      <c r="O13" s="6" t="s">
-        <v>22</v>
+      <c r="O13" s="6">
+        <v>4</v>
       </c>
       <c r="P13" s="6">
-        <v>555</v>
+        <v>617</v>
       </c>
       <c r="Q13" s="6">
-        <v>554</v>
+        <v>492</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Actualizar datos 2026 (2026-04-20)
</commit_message>
<xml_diff>
--- a/data/asistencia/Bravos 2026.xlsx
+++ b/data/asistencia/Bravos 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>51.21%</t>
+    <t>58.45%</t>
   </si>
   <si>
     <t>Butaca 3ra Base</t>
   </si>
   <si>
-    <t>50.19%</t>
+    <t>51.12%</t>
   </si>
   <si>
     <t>General 1ra Base</t>
@@ -100,13 +100,13 @@
     <t>General 3ra Base</t>
   </si>
   <si>
-    <t>3.55%</t>
+    <t>4.23%</t>
   </si>
   <si>
     <t>Parrilladas</t>
   </si>
   <si>
-    <t>0.00%</t>
+    <t>5.56%</t>
   </si>
   <si>
     <t>Personas con Discapacidad</t>
@@ -118,19 +118,19 @@
     <t>VIP</t>
   </si>
   <si>
-    <t>82.88%</t>
+    <t>87.23%</t>
   </si>
   <si>
     <t>Zona Gas Noel Butaca Central</t>
   </si>
   <si>
-    <t>55.64%</t>
+    <t>69.79%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>29.97%</t>
+    <t>34.57%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>828</v>
       </c>
       <c r="C6" s="6">
-        <v>252</v>
+        <v>314</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -676,16 +676,16 @@
         <v>22</v>
       </c>
       <c r="N6" s="6">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>424</v>
+        <v>484</v>
       </c>
       <c r="Q6" s="6">
-        <v>404</v>
+        <v>344</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +699,7 @@
         <v>534</v>
       </c>
       <c r="C7" s="6">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -734,14 +734,14 @@
       <c r="N7" s="6">
         <v>107</v>
       </c>
-      <c r="O7" s="6">
-        <v>7</v>
+      <c r="O7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P7" s="6">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="Q7" s="6">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -811,7 +811,7 @@
         <v>1324</v>
       </c>
       <c r="C9" s="6">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>22</v>
@@ -850,10 +850,10 @@
         <v>22</v>
       </c>
       <c r="P9" s="6">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="Q9" s="6">
-        <v>1277</v>
+        <v>1268</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
@@ -866,8 +866,8 @@
       <c r="B10" s="6">
         <v>180</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>22</v>
+      <c r="C10" s="6">
+        <v>10</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>22</v>
@@ -905,11 +905,11 @@
       <c r="O10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="P10" s="6" t="s">
-        <v>22</v>
+      <c r="P10" s="6">
+        <v>10</v>
       </c>
       <c r="Q10" s="6">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="R10" s="6" t="s">
         <v>31</v>
@@ -979,13 +979,13 @@
         <v>368</v>
       </c>
       <c r="C12" s="6">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
@@ -1012,16 +1012,16 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>305</v>
+        <v>321</v>
       </c>
       <c r="Q12" s="6">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>35</v>
@@ -1035,13 +1035,13 @@
         <v>1109</v>
       </c>
       <c r="C13" s="6">
-        <v>329</v>
+        <v>451</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="6">
-        <v>131</v>
+        <v>164</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>22</v>
@@ -1071,13 +1071,13 @@
         <v>43</v>
       </c>
       <c r="O13" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P13" s="6">
-        <v>617</v>
+        <v>774</v>
       </c>
       <c r="Q13" s="6">
-        <v>492</v>
+        <v>335</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>37</v>

</xml_diff>